<commit_message>
Add Golf Dashboard 2.0 PBIP and documentation
- Created a new PBIP file for Golf Dashboard 2.0, enabling source control for the report.
- Added DASHBOARD_MAP.md to document the structure and navigation of the report, including details on pages, visuals, and data model.
</commit_message>
<xml_diff>
--- a/data/derived/round_profiles.xlsx
+++ b/data/derived/round_profiles.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2122a01115dfea8f/Projects/Golf Stats/data/derived/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_23F921ED8BFB8F2A5B5B3C911CF57D6855941957" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F7AD25D-31DB-417A-8B66-2C8A9FB5D599}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -58,7 +52,7 @@
     <t>z_Irons</t>
   </si>
   <si>
-    <t>z_ShortGame</t>
+    <t>z_Wedges</t>
   </si>
   <si>
     <t>z_Putting</t>
@@ -70,7 +64,7 @@
     <t>Irons</t>
   </si>
   <si>
-    <t>ShortGame</t>
+    <t>Wedges</t>
   </si>
   <si>
     <t>Putting</t>
@@ -166,11 +160,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,21 +228,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -286,7 +272,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -320,7 +306,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -355,10 +340,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -531,30 +515,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:U81"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -619,7 +584,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -630,13 +595,13 @@
         <v>24</v>
       </c>
       <c r="D2">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="E2">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F2">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="G2">
         <v>34</v>
@@ -651,13 +616,13 @@
         <v>12</v>
       </c>
       <c r="K2">
-        <v>2.1999999999999999E-2</v>
+        <v>0.022</v>
       </c>
       <c r="L2">
-        <v>0.76100000000000001</v>
+        <v>0.761</v>
       </c>
       <c r="M2">
-        <v>-8.5999999999999993E-2</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="N2">
         <v>0.311</v>
@@ -684,7 +649,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -695,10 +660,10 @@
         <v>25</v>
       </c>
       <c r="D3">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="E3">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="F3">
         <v>0.1</v>
@@ -716,7 +681,7 @@
         <v>10</v>
       </c>
       <c r="K3">
-        <v>2.1999999999999999E-2</v>
+        <v>0.022</v>
       </c>
       <c r="L3">
         <v>1.518</v>
@@ -725,7 +690,7 @@
         <v>-0.622</v>
       </c>
       <c r="N3">
-        <v>-1.0509999999999999</v>
+        <v>-1.051</v>
       </c>
       <c r="O3" t="s">
         <v>44</v>
@@ -749,7 +714,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -763,7 +728,7 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0.38900000000000001</v>
+        <v>0.389</v>
       </c>
       <c r="G4">
         <v>31</v>
@@ -781,10 +746,10 @@
         <v>-1.508</v>
       </c>
       <c r="M4">
-        <v>1.6990000000000001</v>
+        <v>1.699</v>
       </c>
       <c r="N4">
-        <v>1.3320000000000001</v>
+        <v>1.332</v>
       </c>
       <c r="P4" t="s">
         <v>45</v>
@@ -805,7 +770,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -816,10 +781,10 @@
         <v>27</v>
       </c>
       <c r="D5">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E5">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="F5">
         <v>0.308</v>
@@ -837,16 +802,16 @@
         <v>13</v>
       </c>
       <c r="K5">
-        <v>0.48599999999999999</v>
+        <v>0.486</v>
       </c>
       <c r="L5">
-        <v>0.38300000000000001</v>
+        <v>0.383</v>
       </c>
       <c r="M5">
-        <v>1.0469999999999999</v>
+        <v>1.047</v>
       </c>
       <c r="N5">
-        <v>0.99199999999999999</v>
+        <v>0.992</v>
       </c>
       <c r="O5" t="s">
         <v>44</v>
@@ -870,7 +835,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -884,10 +849,10 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F6">
-        <v>0.17599999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="G6">
         <v>34</v>
@@ -905,10 +870,10 @@
         <v>-1.835</v>
       </c>
       <c r="L6">
-        <v>-1.1299999999999999</v>
+        <v>-1.13</v>
       </c>
       <c r="M6">
-        <v>-7.0000000000000001E-3</v>
+        <v>-0.007</v>
       </c>
       <c r="N6">
         <v>0.311</v>
@@ -935,7 +900,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -946,10 +911,10 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="E7">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="F7">
         <v>0.188</v>
@@ -967,13 +932,13 @@
         <v>16</v>
       </c>
       <c r="K7">
-        <v>-0.90600000000000003</v>
+        <v>-0.906</v>
       </c>
       <c r="L7">
-        <v>-0.53600000000000003</v>
+        <v>-0.536</v>
       </c>
       <c r="M7">
-        <v>8.1000000000000003E-2</v>
+        <v>0.081</v>
       </c>
       <c r="N7">
         <v>0.311</v>
@@ -1000,7 +965,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1011,13 +976,13 @@
         <v>29</v>
       </c>
       <c r="D8">
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="E8">
-        <v>5.8999999999999997E-2</v>
+        <v>0.059</v>
       </c>
       <c r="F8">
-        <v>0.47099999999999997</v>
+        <v>0.471</v>
       </c>
       <c r="G8">
         <v>28</v>
@@ -1032,16 +997,16 @@
         <v>17</v>
       </c>
       <c r="K8">
-        <v>-0.10199999999999999</v>
+        <v>-0.102</v>
       </c>
       <c r="L8">
-        <v>-1.1080000000000001</v>
+        <v>-1.108</v>
       </c>
       <c r="M8">
         <v>2.355</v>
       </c>
       <c r="N8">
-        <v>2.3530000000000002</v>
+        <v>2.353</v>
       </c>
       <c r="O8" t="s">
         <v>44</v>
@@ -1065,7 +1030,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1100,7 +1065,7 @@
         <v>-0.442</v>
       </c>
       <c r="L9">
-        <v>-0.14699999999999999</v>
+        <v>-0.147</v>
       </c>
       <c r="M9">
         <v>-1.425</v>
@@ -1130,7 +1095,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1141,10 +1106,10 @@
         <v>27</v>
       </c>
       <c r="D10">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="E10">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F10">
         <v>0.25</v>
@@ -1162,16 +1127,16 @@
         <v>12</v>
       </c>
       <c r="K10">
-        <v>-0.90600000000000003</v>
+        <v>-0.906</v>
       </c>
       <c r="L10">
-        <v>0.76100000000000001</v>
+        <v>0.761</v>
       </c>
       <c r="M10">
-        <v>0.58299999999999996</v>
+        <v>0.583</v>
       </c>
       <c r="N10">
-        <v>-1.0509999999999999</v>
+        <v>-1.051</v>
       </c>
       <c r="O10" t="s">
         <v>45</v>
@@ -1195,7 +1160,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1209,10 +1174,10 @@
         <v>0.214</v>
       </c>
       <c r="E11">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="F11">
-        <v>6.7000000000000004E-2</v>
+        <v>0.067</v>
       </c>
       <c r="G11">
         <v>37</v>
@@ -1233,7 +1198,7 @@
         <v>-0.374</v>
       </c>
       <c r="M11">
-        <v>-0.88900000000000001</v>
+        <v>-0.889</v>
       </c>
       <c r="N11">
         <v>-0.71</v>
@@ -1260,7 +1225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1325,7 +1290,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1342,7 +1307,7 @@
         <v>0.222</v>
       </c>
       <c r="F13">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="G13">
         <v>36</v>
@@ -1360,10 +1325,10 @@
         <v>-0.442</v>
       </c>
       <c r="L13">
-        <v>5.0000000000000001E-3</v>
+        <v>0.005</v>
       </c>
       <c r="M13">
-        <v>-0.27700000000000002</v>
+        <v>-0.277</v>
       </c>
       <c r="N13">
         <v>-0.37</v>
@@ -1390,7 +1355,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1401,13 +1366,13 @@
         <v>29</v>
       </c>
       <c r="D14">
-        <v>6.7000000000000004E-2</v>
+        <v>0.067</v>
       </c>
       <c r="E14">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F14">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="G14">
         <v>34</v>
@@ -1425,10 +1390,10 @@
         <v>-1.401</v>
       </c>
       <c r="L14">
-        <v>0.76100000000000001</v>
+        <v>0.761</v>
       </c>
       <c r="M14">
-        <v>-8.5999999999999993E-2</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="N14">
         <v>0.311</v>
@@ -1455,7 +1420,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1466,13 +1431,13 @@
         <v>27</v>
       </c>
       <c r="D15">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E15">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="F15">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="G15">
         <v>31</v>
@@ -1496,7 +1461,7 @@
         <v>1.252</v>
       </c>
       <c r="N15">
-        <v>1.3320000000000001</v>
+        <v>1.332</v>
       </c>
       <c r="O15" t="s">
         <v>46</v>
@@ -1520,7 +1485,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1531,10 +1496,10 @@
         <v>27</v>
       </c>
       <c r="D16">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E16">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="F16">
         <v>0.1</v>
@@ -1585,7 +1550,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1596,10 +1561,10 @@
         <v>33</v>
       </c>
       <c r="D17">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E17">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="F17">
         <v>0.1</v>
@@ -1617,7 +1582,7 @@
         <v>10</v>
       </c>
       <c r="K17">
-        <v>1.8779999999999999</v>
+        <v>1.878</v>
       </c>
       <c r="L17">
         <v>1.518</v>
@@ -1650,7 +1615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1661,13 +1626,13 @@
         <v>33</v>
       </c>
       <c r="D18">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E18">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F18">
-        <v>8.3000000000000004E-2</v>
+        <v>0.083</v>
       </c>
       <c r="G18">
         <v>38</v>
@@ -1682,16 +1647,16 @@
         <v>12</v>
       </c>
       <c r="K18">
-        <v>1.8779999999999999</v>
+        <v>1.878</v>
       </c>
       <c r="L18">
-        <v>0.76100000000000001</v>
+        <v>0.761</v>
       </c>
       <c r="M18">
-        <v>-0.75600000000000001</v>
+        <v>-0.756</v>
       </c>
       <c r="N18">
-        <v>-1.0509999999999999</v>
+        <v>-1.051</v>
       </c>
       <c r="O18" t="s">
         <v>46</v>
@@ -1715,7 +1680,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1726,7 +1691,7 @@
         <v>33</v>
       </c>
       <c r="D19">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -1747,7 +1712,7 @@
         <v>18</v>
       </c>
       <c r="K19">
-        <v>0.48599999999999999</v>
+        <v>0.486</v>
       </c>
       <c r="L19">
         <v>-1.508</v>
@@ -1756,7 +1721,7 @@
         <v>0.36</v>
       </c>
       <c r="N19">
-        <v>0.99199999999999999</v>
+        <v>0.992</v>
       </c>
       <c r="O19" t="s">
         <v>44</v>
@@ -1780,7 +1745,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1794,10 +1759,10 @@
         <v>0.5</v>
       </c>
       <c r="E20">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F20">
-        <v>0.29399999999999998</v>
+        <v>0.294</v>
       </c>
       <c r="G20">
         <v>33</v>
@@ -1812,16 +1777,16 @@
         <v>17</v>
       </c>
       <c r="K20">
-        <v>1.4139999999999999</v>
+        <v>1.414</v>
       </c>
       <c r="L20">
-        <v>-1.1299999999999999</v>
+        <v>-1.13</v>
       </c>
       <c r="M20">
-        <v>0.93700000000000006</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="N20">
-        <v>0.65100000000000002</v>
+        <v>0.651</v>
       </c>
       <c r="O20" t="s">
         <v>46</v>
@@ -1845,7 +1810,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1856,13 +1821,13 @@
         <v>27</v>
       </c>
       <c r="D21">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="E21">
-        <v>9.0999999999999998E-2</v>
+        <v>0.091</v>
       </c>
       <c r="F21">
-        <v>0.29399999999999998</v>
+        <v>0.294</v>
       </c>
       <c r="G21">
         <v>33</v>
@@ -1877,16 +1842,16 @@
         <v>17</v>
       </c>
       <c r="K21">
-        <v>-0.90600000000000003</v>
+        <v>-0.906</v>
       </c>
       <c r="L21">
-        <v>-0.88900000000000001</v>
+        <v>-0.889</v>
       </c>
       <c r="M21">
-        <v>0.93700000000000006</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="N21">
-        <v>0.65100000000000002</v>
+        <v>0.651</v>
       </c>
       <c r="O21" t="s">
         <v>45</v>
@@ -1910,7 +1875,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1921,13 +1886,13 @@
         <v>33</v>
       </c>
       <c r="D22">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="E22">
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="F22">
-        <v>7.0999999999999994E-2</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G22">
         <v>37</v>
@@ -1942,13 +1907,13 @@
         <v>14</v>
       </c>
       <c r="K22">
-        <v>-0.90600000000000003</v>
+        <v>-0.906</v>
       </c>
       <c r="L22">
         <v>0.307</v>
       </c>
       <c r="M22">
-        <v>-0.85099999999999998</v>
+        <v>-0.851</v>
       </c>
       <c r="N22">
         <v>-0.71</v>
@@ -1975,7 +1940,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1992,7 +1957,7 @@
         <v>0.438</v>
       </c>
       <c r="F23">
-        <v>9.0999999999999998E-2</v>
+        <v>0.091</v>
       </c>
       <c r="G23">
         <v>39</v>
@@ -2007,13 +1972,13 @@
         <v>11</v>
       </c>
       <c r="K23">
-        <v>0.16400000000000001</v>
+        <v>0.164</v>
       </c>
       <c r="L23">
         <v>1.47</v>
       </c>
       <c r="M23">
-        <v>-0.69499999999999995</v>
+        <v>-0.695</v>
       </c>
       <c r="N23">
         <v>-1.391</v>
@@ -2040,7 +2005,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -2051,13 +2016,13 @@
         <v>35</v>
       </c>
       <c r="D24">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E24">
-        <v>0.17599999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="F24">
-        <v>6.7000000000000004E-2</v>
+        <v>0.067</v>
       </c>
       <c r="G24">
         <v>38</v>
@@ -2072,16 +2037,16 @@
         <v>15</v>
       </c>
       <c r="K24">
-        <v>0.48599999999999999</v>
+        <v>0.486</v>
       </c>
       <c r="L24">
         <v>-0.307</v>
       </c>
       <c r="M24">
-        <v>-0.88900000000000001</v>
+        <v>-0.889</v>
       </c>
       <c r="N24">
-        <v>-1.0509999999999999</v>
+        <v>-1.051</v>
       </c>
       <c r="O24" t="s">
         <v>44</v>
@@ -2105,7 +2070,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2119,10 +2084,10 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F25">
-        <v>0.17599999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="G25">
         <v>35</v>
@@ -2137,16 +2102,16 @@
         <v>17</v>
       </c>
       <c r="K25">
-        <v>-1.5820000000000001</v>
+        <v>-1.582</v>
       </c>
       <c r="L25">
-        <v>-1.2470000000000001</v>
+        <v>-1.247</v>
       </c>
       <c r="M25">
         <v>0.434</v>
       </c>
       <c r="N25">
-        <v>0.93600000000000005</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="O25" t="s">
         <v>45</v>
@@ -2170,7 +2135,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21">
       <c r="A26" t="s">
         <v>22</v>
       </c>
@@ -2181,13 +2146,13 @@
         <v>29</v>
       </c>
       <c r="D26">
-        <v>0.46700000000000003</v>
+        <v>0.467</v>
       </c>
       <c r="E26">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F26">
-        <v>0.17599999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="G26">
         <v>34</v>
@@ -2202,10 +2167,10 @@
         <v>17</v>
       </c>
       <c r="K26">
-        <v>0.89600000000000002</v>
+        <v>0.896</v>
       </c>
       <c r="L26">
-        <v>-1.2470000000000001</v>
+        <v>-1.247</v>
       </c>
       <c r="M26">
         <v>0.434</v>
@@ -2235,7 +2200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21">
       <c r="A27" t="s">
         <v>22</v>
       </c>
@@ -2252,7 +2217,7 @@
         <v>0.222</v>
       </c>
       <c r="F27">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="G27">
         <v>36</v>
@@ -2267,16 +2232,16 @@
         <v>14</v>
       </c>
       <c r="K27">
-        <v>1.0740000000000001</v>
+        <v>1.074</v>
       </c>
       <c r="L27">
-        <v>1.2589999999999999</v>
+        <v>1.259</v>
       </c>
       <c r="M27">
-        <v>0.14199999999999999</v>
+        <v>0.142</v>
       </c>
       <c r="N27">
-        <v>0.72599999999999998</v>
+        <v>0.726</v>
       </c>
       <c r="O27" t="s">
         <v>46</v>
@@ -2300,7 +2265,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2311,7 +2276,7 @@
         <v>37</v>
       </c>
       <c r="D28">
-        <v>0.38500000000000001</v>
+        <v>0.385</v>
       </c>
       <c r="E28">
         <v>0.125</v>
@@ -2332,16 +2297,16 @@
         <v>16</v>
       </c>
       <c r="K28">
-        <v>0.46100000000000002</v>
+        <v>0.461</v>
       </c>
       <c r="L28">
-        <v>-0.20300000000000001</v>
+        <v>-0.203</v>
       </c>
       <c r="M28">
-        <v>-1.0980000000000001</v>
+        <v>-1.098</v>
       </c>
       <c r="N28">
-        <v>-0.53800000000000003</v>
+        <v>-0.538</v>
       </c>
       <c r="O28" t="s">
         <v>44</v>
@@ -2365,7 +2330,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -2397,13 +2362,13 @@
         <v>16</v>
       </c>
       <c r="K29">
-        <v>-1.5820000000000001</v>
+        <v>-1.582</v>
       </c>
       <c r="L29">
-        <v>-0.41199999999999998</v>
+        <v>-0.412</v>
       </c>
       <c r="M29">
-        <v>-1.0980000000000001</v>
+        <v>-1.098</v>
       </c>
       <c r="N29">
         <v>-1.17</v>
@@ -2430,7 +2395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -2441,13 +2406,13 @@
         <v>36</v>
       </c>
       <c r="D30">
-        <v>0.23100000000000001</v>
+        <v>0.231</v>
       </c>
       <c r="E30">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="F30">
-        <v>0.13300000000000001</v>
+        <v>0.133</v>
       </c>
       <c r="G30">
         <v>42</v>
@@ -2462,16 +2427,16 @@
         <v>15</v>
       </c>
       <c r="K30">
-        <v>-0.35599999999999998</v>
+        <v>-0.356</v>
       </c>
       <c r="L30">
-        <v>0.42299999999999999</v>
+        <v>0.423</v>
       </c>
       <c r="M30">
         <v>0.06</v>
       </c>
       <c r="N30">
-        <v>-0.53800000000000003</v>
+        <v>-0.538</v>
       </c>
       <c r="O30" t="s">
         <v>44</v>
@@ -2495,7 +2460,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21">
       <c r="A31" t="s">
         <v>22</v>
       </c>
@@ -2506,13 +2471,13 @@
         <v>39</v>
       </c>
       <c r="D31">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="E31">
         <v>0.25</v>
       </c>
       <c r="F31">
-        <v>7.0999999999999994E-2</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G31">
         <v>41</v>
@@ -2527,16 +2492,16 @@
         <v>14</v>
       </c>
       <c r="K31">
-        <v>-6.5000000000000002E-2</v>
+        <v>-0.065</v>
       </c>
       <c r="L31">
-        <v>1.6759999999999999</v>
+        <v>1.676</v>
       </c>
       <c r="M31">
-        <v>-0.47799999999999998</v>
+        <v>-0.478</v>
       </c>
       <c r="N31">
-        <v>-0.32800000000000001</v>
+        <v>-0.328</v>
       </c>
       <c r="O31" t="s">
         <v>44</v>
@@ -2560,7 +2525,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -2571,10 +2536,10 @@
         <v>36</v>
       </c>
       <c r="D32">
-        <v>0.38500000000000001</v>
+        <v>0.385</v>
       </c>
       <c r="E32">
-        <v>0.11799999999999999</v>
+        <v>0.118</v>
       </c>
       <c r="F32">
         <v>0.375</v>
@@ -2592,7 +2557,7 @@
         <v>16</v>
       </c>
       <c r="K32">
-        <v>0.46100000000000002</v>
+        <v>0.461</v>
       </c>
       <c r="L32">
         <v>-0.314</v>
@@ -2625,7 +2590,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -2636,13 +2601,13 @@
         <v>40</v>
       </c>
       <c r="D33">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E33">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="F33">
-        <v>6.2E-2</v>
+        <v>0.062</v>
       </c>
       <c r="G33">
         <v>46</v>
@@ -2657,13 +2622,13 @@
         <v>16</v>
       </c>
       <c r="K33">
-        <v>0.69399999999999995</v>
+        <v>0.694</v>
       </c>
       <c r="L33">
-        <v>6.5000000000000002E-2</v>
+        <v>0.065</v>
       </c>
       <c r="M33">
-        <v>-0.55500000000000005</v>
+        <v>-0.555</v>
       </c>
       <c r="N33">
         <v>-1.381</v>
@@ -2690,7 +2655,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -2701,13 +2666,13 @@
         <v>24</v>
       </c>
       <c r="D34">
-        <v>0.64300000000000002</v>
+        <v>0.643</v>
       </c>
       <c r="E34">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="F34">
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="G34">
         <v>36</v>
@@ -2722,10 +2687,10 @@
         <v>15</v>
       </c>
       <c r="K34">
-        <v>1.1879999999999999</v>
+        <v>1.188</v>
       </c>
       <c r="L34">
-        <v>-0.74099999999999999</v>
+        <v>-0.741</v>
       </c>
       <c r="M34">
         <v>-0.216</v>
@@ -2755,7 +2720,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -2772,7 +2737,7 @@
         <v>0.222</v>
       </c>
       <c r="F35">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="G35">
         <v>37</v>
@@ -2787,7 +2752,7 @@
         <v>14</v>
       </c>
       <c r="K35">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L35">
         <v>-0.38</v>
@@ -2796,7 +2761,7 @@
         <v>-1.022</v>
       </c>
       <c r="N35">
-        <v>-1.3089999999999999</v>
+        <v>-1.309</v>
       </c>
       <c r="O35" t="s">
         <v>44</v>
@@ -2820,7 +2785,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -2837,7 +2802,7 @@
         <v>0.222</v>
       </c>
       <c r="F36">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="G36">
         <v>37</v>
@@ -2852,7 +2817,7 @@
         <v>14</v>
       </c>
       <c r="K36">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L36">
         <v>-0.38</v>
@@ -2861,7 +2826,7 @@
         <v>-1.022</v>
       </c>
       <c r="N36">
-        <v>-1.3089999999999999</v>
+        <v>-1.309</v>
       </c>
       <c r="O36" t="s">
         <v>44</v>
@@ -2885,7 +2850,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -2896,7 +2861,7 @@
         <v>25</v>
       </c>
       <c r="D37">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E37">
         <v>0.111</v>
@@ -2917,13 +2882,13 @@
         <v>16</v>
       </c>
       <c r="K37">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L37">
         <v>-1.101</v>
       </c>
       <c r="M37">
-        <v>-0.32500000000000001</v>
+        <v>-0.325</v>
       </c>
       <c r="N37">
         <v>-0.996</v>
@@ -2950,7 +2915,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21">
       <c r="A38" t="s">
         <v>23</v>
       </c>
@@ -2961,7 +2926,7 @@
         <v>24</v>
       </c>
       <c r="D38">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E38">
         <v>0.111</v>
@@ -2982,16 +2947,16 @@
         <v>16</v>
       </c>
       <c r="K38">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L38">
         <v>-1.101</v>
       </c>
       <c r="M38">
-        <v>-0.73099999999999998</v>
+        <v>-0.731</v>
       </c>
       <c r="N38">
-        <v>-1.3089999999999999</v>
+        <v>-1.309</v>
       </c>
       <c r="O38" t="s">
         <v>44</v>
@@ -3015,7 +2980,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21">
       <c r="A39" t="s">
         <v>23</v>
       </c>
@@ -3026,7 +2991,7 @@
         <v>25</v>
       </c>
       <c r="D39">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="E39">
         <v>0.222</v>
@@ -3047,13 +3012,13 @@
         <v>14</v>
       </c>
       <c r="K39">
-        <v>-1.1890000000000001</v>
+        <v>-1.189</v>
       </c>
       <c r="L39">
         <v>-0.38</v>
       </c>
       <c r="M39">
-        <v>-0.55700000000000005</v>
+        <v>-0.5570000000000001</v>
       </c>
       <c r="N39">
         <v>0.254</v>
@@ -3080,7 +3045,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21">
       <c r="A40" t="s">
         <v>23</v>
       </c>
@@ -3091,10 +3056,10 @@
         <v>25</v>
       </c>
       <c r="D40">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E40">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -3112,16 +3077,16 @@
         <v>13</v>
       </c>
       <c r="K40">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L40">
         <v>-0.02</v>
       </c>
       <c r="M40">
-        <v>-1.9510000000000001</v>
+        <v>-1.951</v>
       </c>
       <c r="N40">
-        <v>-1.9339999999999999</v>
+        <v>-1.934</v>
       </c>
       <c r="O40" t="s">
         <v>44</v>
@@ -3145,7 +3110,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21">
       <c r="A41" t="s">
         <v>23</v>
       </c>
@@ -3156,13 +3121,13 @@
         <v>41</v>
       </c>
       <c r="D41">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E41">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F41">
-        <v>0.35299999999999998</v>
+        <v>0.353</v>
       </c>
       <c r="G41">
         <v>32</v>
@@ -3177,13 +3142,13 @@
         <v>17</v>
       </c>
       <c r="K41">
-        <v>0.71199999999999997</v>
+        <v>0.712</v>
       </c>
       <c r="L41">
-        <v>-1.4610000000000001</v>
+        <v>-1.461</v>
       </c>
       <c r="M41">
-        <v>0.34499999999999997</v>
+        <v>0.345</v>
       </c>
       <c r="N41">
         <v>0.254</v>
@@ -3210,7 +3175,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21">
       <c r="A42" t="s">
         <v>23</v>
       </c>
@@ -3221,13 +3186,13 @@
         <v>26</v>
       </c>
       <c r="D42">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E42">
         <v>0.222</v>
       </c>
       <c r="F42">
-        <v>7.0999999999999994E-2</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G42">
         <v>35</v>
@@ -3242,16 +3207,16 @@
         <v>14</v>
       </c>
       <c r="K42">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L42">
         <v>-0.38</v>
       </c>
       <c r="M42">
-        <v>-1.4870000000000001</v>
+        <v>-1.487</v>
       </c>
       <c r="N42">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O42" t="s">
         <v>44</v>
@@ -3275,7 +3240,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21">
       <c r="A43" t="s">
         <v>23</v>
       </c>
@@ -3286,13 +3251,13 @@
         <v>27</v>
       </c>
       <c r="D43">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E43">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F43">
-        <v>8.3000000000000004E-2</v>
+        <v>0.083</v>
       </c>
       <c r="G43">
         <v>37</v>
@@ -3307,7 +3272,7 @@
         <v>12</v>
       </c>
       <c r="K43">
-        <v>0.71199999999999997</v>
+        <v>0.712</v>
       </c>
       <c r="L43">
         <v>0.34</v>
@@ -3316,7 +3281,7 @@
         <v>-1.409</v>
       </c>
       <c r="N43">
-        <v>-1.3089999999999999</v>
+        <v>-1.309</v>
       </c>
       <c r="O43" t="s">
         <v>46</v>
@@ -3340,7 +3305,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21">
       <c r="A44" t="s">
         <v>23</v>
       </c>
@@ -3354,10 +3319,10 @@
         <v>0.214</v>
       </c>
       <c r="E44">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F44">
-        <v>8.3000000000000004E-2</v>
+        <v>0.083</v>
       </c>
       <c r="G44">
         <v>38</v>
@@ -3405,7 +3370,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21">
       <c r="A45" t="s">
         <v>23</v>
       </c>
@@ -3437,16 +3402,16 @@
         <v>16</v>
       </c>
       <c r="K45">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L45">
         <v>-1.101</v>
       </c>
       <c r="M45">
-        <v>-0.32500000000000001</v>
+        <v>-0.325</v>
       </c>
       <c r="N45">
-        <v>-5.8999999999999997E-2</v>
+        <v>-0.059</v>
       </c>
       <c r="O45" t="s">
         <v>44</v>
@@ -3470,7 +3435,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21">
       <c r="A46" t="s">
         <v>23</v>
       </c>
@@ -3481,13 +3446,13 @@
         <v>27</v>
       </c>
       <c r="D46">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="E46">
         <v>0.375</v>
       </c>
       <c r="F46">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="G46">
         <v>35</v>
@@ -3502,16 +3467,16 @@
         <v>12</v>
       </c>
       <c r="K46">
-        <v>-1.1890000000000001</v>
+        <v>-1.189</v>
       </c>
       <c r="L46">
         <v>0.61</v>
       </c>
       <c r="M46">
-        <v>-0.86699999999999999</v>
+        <v>-0.867</v>
       </c>
       <c r="N46">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O46" t="s">
         <v>45</v>
@@ -3535,7 +3500,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21">
       <c r="A47" t="s">
         <v>23</v>
       </c>
@@ -3546,13 +3511,13 @@
         <v>36</v>
       </c>
       <c r="D47">
-        <v>0.38500000000000001</v>
+        <v>0.385</v>
       </c>
       <c r="E47">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="F47">
-        <v>0.13300000000000001</v>
+        <v>0.133</v>
       </c>
       <c r="G47">
         <v>35</v>
@@ -3567,16 +3532,16 @@
         <v>15</v>
       </c>
       <c r="K47">
-        <v>-0.53100000000000003</v>
+        <v>-0.531</v>
       </c>
       <c r="L47">
-        <v>-0.74099999999999999</v>
+        <v>-0.741</v>
       </c>
       <c r="M47">
-        <v>-1.0840000000000001</v>
+        <v>-1.084</v>
       </c>
       <c r="N47">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O47" t="s">
         <v>45</v>
@@ -3600,7 +3565,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21">
       <c r="A48" t="s">
         <v>23</v>
       </c>
@@ -3638,10 +3603,10 @@
         <v>-1.101</v>
       </c>
       <c r="M48">
-        <v>-0.73099999999999998</v>
+        <v>-0.731</v>
       </c>
       <c r="N48">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O48" t="s">
         <v>45</v>
@@ -3665,7 +3630,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21">
       <c r="A49" t="s">
         <v>23</v>
       </c>
@@ -3682,7 +3647,7 @@
         <v>0.222</v>
       </c>
       <c r="F49">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="G49">
         <v>30</v>
@@ -3697,13 +3662,13 @@
         <v>14</v>
       </c>
       <c r="K49">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L49">
         <v>-0.38</v>
       </c>
       <c r="M49">
-        <v>0.83699999999999997</v>
+        <v>0.837</v>
       </c>
       <c r="N49">
         <v>0.879</v>
@@ -3730,7 +3695,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21">
       <c r="A50" t="s">
         <v>23</v>
       </c>
@@ -3741,13 +3706,13 @@
         <v>24</v>
       </c>
       <c r="D50">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E50">
-        <v>0.69199999999999995</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F50">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="G50">
         <v>33</v>
@@ -3762,16 +3727,16 @@
         <v>9</v>
       </c>
       <c r="K50">
-        <v>-0.71399999999999997</v>
+        <v>-0.714</v>
       </c>
       <c r="L50">
-        <v>2.6680000000000001</v>
+        <v>2.668</v>
       </c>
       <c r="M50">
         <v>0.218</v>
       </c>
       <c r="N50">
-        <v>-5.8999999999999997E-2</v>
+        <v>-0.059</v>
       </c>
       <c r="O50" t="s">
         <v>45</v>
@@ -3795,7 +3760,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21">
       <c r="A51" t="s">
         <v>23</v>
       </c>
@@ -3806,10 +3771,10 @@
         <v>24</v>
       </c>
       <c r="D51">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E51">
-        <v>0.53300000000000003</v>
+        <v>0.533</v>
       </c>
       <c r="F51">
         <v>0.5</v>
@@ -3827,7 +3792,7 @@
         <v>10</v>
       </c>
       <c r="K51">
-        <v>0.71199999999999997</v>
+        <v>0.712</v>
       </c>
       <c r="L51">
         <v>1.637</v>
@@ -3836,7 +3801,7 @@
         <v>1.302</v>
       </c>
       <c r="N51">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O51" t="s">
         <v>46</v>
@@ -3860,7 +3825,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21">
       <c r="A52" t="s">
         <v>23</v>
       </c>
@@ -3871,7 +3836,7 @@
         <v>42</v>
       </c>
       <c r="D52">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E52">
         <v>0.111</v>
@@ -3892,13 +3857,13 @@
         <v>16</v>
       </c>
       <c r="K52">
-        <v>0.71199999999999997</v>
+        <v>0.712</v>
       </c>
       <c r="L52">
         <v>-1.101</v>
       </c>
       <c r="M52">
-        <v>0.48899999999999999</v>
+        <v>0.489</v>
       </c>
       <c r="N52">
         <v>0.879</v>
@@ -3925,7 +3890,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21">
       <c r="A53" t="s">
         <v>23</v>
       </c>
@@ -3939,7 +3904,7 @@
         <v>0.214</v>
       </c>
       <c r="E53">
-        <v>0.35299999999999998</v>
+        <v>0.353</v>
       </c>
       <c r="F53">
         <v>0.5</v>
@@ -3960,13 +3925,13 @@
         <v>-1.665</v>
       </c>
       <c r="L53">
-        <v>0.46700000000000003</v>
+        <v>0.467</v>
       </c>
       <c r="M53">
         <v>1.302</v>
       </c>
       <c r="N53">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O53" t="s">
         <v>45</v>
@@ -3990,7 +3955,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21">
       <c r="A54" t="s">
         <v>23</v>
       </c>
@@ -4001,13 +3966,13 @@
         <v>29</v>
       </c>
       <c r="D54">
-        <v>0.53300000000000003</v>
+        <v>0.533</v>
       </c>
       <c r="E54">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="F54">
-        <v>0.46200000000000002</v>
+        <v>0.462</v>
       </c>
       <c r="G54">
         <v>29</v>
@@ -4022,7 +3987,7 @@
         <v>13</v>
       </c>
       <c r="K54">
-        <v>0.45900000000000002</v>
+        <v>0.459</v>
       </c>
       <c r="L54">
         <v>-0.02</v>
@@ -4031,7 +3996,7 @@
         <v>1.052</v>
       </c>
       <c r="N54">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O54" t="s">
         <v>44</v>
@@ -4055,7 +4020,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21">
       <c r="A55" t="s">
         <v>23</v>
       </c>
@@ -4069,10 +4034,10 @@
         <v>0.6</v>
       </c>
       <c r="E55">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="F55">
-        <v>0.46700000000000003</v>
+        <v>0.467</v>
       </c>
       <c r="G55">
         <v>27</v>
@@ -4087,16 +4052,16 @@
         <v>15</v>
       </c>
       <c r="K55">
-        <v>0.90300000000000002</v>
+        <v>0.903</v>
       </c>
       <c r="L55">
-        <v>-0.74099999999999999</v>
+        <v>-0.741</v>
       </c>
       <c r="M55">
         <v>1.085</v>
       </c>
       <c r="N55">
-        <v>1.8160000000000001</v>
+        <v>1.816</v>
       </c>
       <c r="O55" t="s">
         <v>46</v>
@@ -4120,7 +4085,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21">
       <c r="A56" t="s">
         <v>23</v>
       </c>
@@ -4131,7 +4096,7 @@
         <v>27</v>
       </c>
       <c r="D56">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E56">
         <v>0.222</v>
@@ -4152,7 +4117,7 @@
         <v>14</v>
       </c>
       <c r="K56">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L56">
         <v>-0.38</v>
@@ -4161,7 +4126,7 @@
         <v>1.302</v>
       </c>
       <c r="N56">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O56" t="s">
         <v>44</v>
@@ -4185,7 +4150,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21">
       <c r="A57" t="s">
         <v>23</v>
       </c>
@@ -4199,7 +4164,7 @@
         <v>0.4</v>
       </c>
       <c r="E57">
-        <v>0.23499999999999999</v>
+        <v>0.235</v>
       </c>
       <c r="F57">
         <v>0.214</v>
@@ -4217,16 +4182,16 @@
         <v>14</v>
       </c>
       <c r="K57">
-        <v>-0.42899999999999999</v>
+        <v>-0.429</v>
       </c>
       <c r="L57">
-        <v>-0.29599999999999999</v>
+        <v>-0.296</v>
       </c>
       <c r="M57">
-        <v>-0.55700000000000005</v>
+        <v>-0.5570000000000001</v>
       </c>
       <c r="N57">
-        <v>0.56599999999999995</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="O57" t="s">
         <v>44</v>
@@ -4250,7 +4215,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21">
       <c r="A58" t="s">
         <v>23</v>
       </c>
@@ -4261,13 +4226,13 @@
         <v>25</v>
       </c>
       <c r="D58">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E58">
-        <v>0.23100000000000001</v>
+        <v>0.231</v>
       </c>
       <c r="F58">
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="G58">
         <v>32</v>
@@ -4282,10 +4247,10 @@
         <v>15</v>
       </c>
       <c r="K58">
-        <v>-0.71399999999999997</v>
+        <v>-0.714</v>
       </c>
       <c r="L58">
-        <v>-0.32500000000000001</v>
+        <v>-0.325</v>
       </c>
       <c r="M58">
         <v>-0.216</v>
@@ -4315,7 +4280,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21">
       <c r="A59" t="s">
         <v>23</v>
       </c>
@@ -4326,13 +4291,13 @@
         <v>27</v>
       </c>
       <c r="D59">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E59">
         <v>0.222</v>
       </c>
       <c r="F59">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="G59">
         <v>29</v>
@@ -4347,7 +4312,7 @@
         <v>14</v>
       </c>
       <c r="K59">
-        <v>-0.71399999999999997</v>
+        <v>-0.714</v>
       </c>
       <c r="L59">
         <v>-0.38</v>
@@ -4356,7 +4321,7 @@
         <v>0.373</v>
       </c>
       <c r="N59">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O59" t="s">
         <v>45</v>
@@ -4380,7 +4345,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21">
       <c r="A60" t="s">
         <v>23</v>
       </c>
@@ -4391,13 +4356,13 @@
         <v>43</v>
       </c>
       <c r="D60">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E60">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="F60">
-        <v>0.46200000000000002</v>
+        <v>0.462</v>
       </c>
       <c r="G60">
         <v>29</v>
@@ -4412,7 +4377,7 @@
         <v>13</v>
       </c>
       <c r="K60">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L60">
         <v>-0.02</v>
@@ -4421,7 +4386,7 @@
         <v>1.052</v>
       </c>
       <c r="N60">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O60" t="s">
         <v>44</v>
@@ -4445,7 +4410,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21">
       <c r="A61" t="s">
         <v>23</v>
       </c>
@@ -4456,13 +4421,13 @@
         <v>30</v>
       </c>
       <c r="D61">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E61">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F61">
-        <v>0.11799999999999999</v>
+        <v>0.118</v>
       </c>
       <c r="G61">
         <v>35</v>
@@ -4477,16 +4442,16 @@
         <v>17</v>
       </c>
       <c r="K61">
-        <v>-0.71399999999999997</v>
+        <v>-0.714</v>
       </c>
       <c r="L61">
-        <v>-1.4610000000000001</v>
+        <v>-1.461</v>
       </c>
       <c r="M61">
-        <v>-1.1859999999999999</v>
+        <v>-1.186</v>
       </c>
       <c r="N61">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O61" t="s">
         <v>45</v>
@@ -4510,7 +4475,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21">
       <c r="A62" t="s">
         <v>23</v>
       </c>
@@ -4521,13 +4486,13 @@
         <v>31</v>
       </c>
       <c r="D62">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E62">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="F62">
-        <v>0.46200000000000002</v>
+        <v>0.462</v>
       </c>
       <c r="G62">
         <v>31</v>
@@ -4542,7 +4507,7 @@
         <v>13</v>
       </c>
       <c r="K62">
-        <v>0.71199999999999997</v>
+        <v>0.712</v>
       </c>
       <c r="L62">
         <v>-0.02</v>
@@ -4551,7 +4516,7 @@
         <v>1.052</v>
       </c>
       <c r="N62">
-        <v>0.56599999999999995</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="O62" t="s">
         <v>46</v>
@@ -4575,7 +4540,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21">
       <c r="A63" t="s">
         <v>23</v>
       </c>
@@ -4586,10 +4551,10 @@
         <v>32</v>
       </c>
       <c r="D63">
-        <v>0.78600000000000003</v>
+        <v>0.786</v>
       </c>
       <c r="E63">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F63">
         <v>0.25</v>
@@ -4607,13 +4572,13 @@
         <v>12</v>
       </c>
       <c r="K63">
-        <v>2.1389999999999998</v>
+        <v>2.139</v>
       </c>
       <c r="L63">
         <v>0.34</v>
       </c>
       <c r="M63">
-        <v>-0.32500000000000001</v>
+        <v>-0.325</v>
       </c>
       <c r="N63">
         <v>-0.371</v>
@@ -4640,7 +4605,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21">
       <c r="A64" t="s">
         <v>23</v>
       </c>
@@ -4654,7 +4619,7 @@
         <v>0.5</v>
       </c>
       <c r="E64">
-        <v>0.55600000000000005</v>
+        <v>0.556</v>
       </c>
       <c r="F64">
         <v>0.5</v>
@@ -4672,16 +4637,16 @@
         <v>8</v>
       </c>
       <c r="K64">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L64">
-        <v>1.7809999999999999</v>
+        <v>1.781</v>
       </c>
       <c r="M64">
         <v>1.302</v>
       </c>
       <c r="N64">
-        <v>0.56599999999999995</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="O64" t="s">
         <v>44</v>
@@ -4705,7 +4670,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21">
       <c r="A65" t="s">
         <v>23</v>
       </c>
@@ -4719,10 +4684,10 @@
         <v>0.6</v>
       </c>
       <c r="E65">
-        <v>0.38900000000000001</v>
+        <v>0.389</v>
       </c>
       <c r="F65">
-        <v>0.54500000000000004</v>
+        <v>0.545</v>
       </c>
       <c r="G65">
         <v>28</v>
@@ -4737,13 +4702,13 @@
         <v>11</v>
       </c>
       <c r="K65">
-        <v>0.90300000000000002</v>
+        <v>0.903</v>
       </c>
       <c r="L65">
         <v>0.7</v>
       </c>
       <c r="M65">
-        <v>1.5980000000000001</v>
+        <v>1.598</v>
       </c>
       <c r="N65">
         <v>1.504</v>
@@ -4770,7 +4735,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21">
       <c r="A66" t="s">
         <v>23</v>
       </c>
@@ -4781,7 +4746,7 @@
         <v>24</v>
       </c>
       <c r="D66">
-        <v>0.57099999999999995</v>
+        <v>0.571</v>
       </c>
       <c r="E66">
         <v>0.5</v>
@@ -4802,7 +4767,7 @@
         <v>9</v>
       </c>
       <c r="K66">
-        <v>0.71199999999999997</v>
+        <v>0.712</v>
       </c>
       <c r="L66">
         <v>1.421</v>
@@ -4835,7 +4800,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21">
       <c r="A67" t="s">
         <v>23</v>
       </c>
@@ -4849,7 +4814,7 @@
         <v>0.5</v>
       </c>
       <c r="E67">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="F67">
         <v>0.4</v>
@@ -4867,13 +4832,13 @@
         <v>10</v>
       </c>
       <c r="K67">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L67">
-        <v>1.0609999999999999</v>
+        <v>1.061</v>
       </c>
       <c r="M67">
-        <v>0.65100000000000002</v>
+        <v>0.651</v>
       </c>
       <c r="N67">
         <v>0.254</v>
@@ -4900,7 +4865,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21">
       <c r="A68" t="s">
         <v>23</v>
       </c>
@@ -4911,13 +4876,13 @@
         <v>27</v>
       </c>
       <c r="D68">
-        <v>0.64300000000000002</v>
+        <v>0.643</v>
       </c>
       <c r="E68">
-        <v>0.61099999999999999</v>
+        <v>0.611</v>
       </c>
       <c r="F68">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="G68">
         <v>33</v>
@@ -4932,16 +4897,16 @@
         <v>7</v>
       </c>
       <c r="K68">
-        <v>1.1879999999999999</v>
+        <v>1.188</v>
       </c>
       <c r="L68">
         <v>2.141</v>
       </c>
       <c r="M68">
-        <v>0.83699999999999997</v>
+        <v>0.837</v>
       </c>
       <c r="N68">
-        <v>-5.8999999999999997E-2</v>
+        <v>-0.059</v>
       </c>
       <c r="O68" t="s">
         <v>46</v>
@@ -4965,7 +4930,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21">
       <c r="A69" t="s">
         <v>23</v>
       </c>
@@ -4997,7 +4962,7 @@
         <v>14</v>
       </c>
       <c r="K69">
-        <v>0.23699999999999999</v>
+        <v>0.237</v>
       </c>
       <c r="L69">
         <v>-0.38</v>
@@ -5006,7 +4971,7 @@
         <v>1.302</v>
       </c>
       <c r="N69">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O69" t="s">
         <v>44</v>
@@ -5030,7 +4995,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:21">
       <c r="A70" t="s">
         <v>23</v>
       </c>
@@ -5041,7 +5006,7 @@
         <v>33</v>
       </c>
       <c r="D70">
-        <v>0.78600000000000003</v>
+        <v>0.786</v>
       </c>
       <c r="E70">
         <v>0.222</v>
@@ -5062,7 +5027,7 @@
         <v>14</v>
       </c>
       <c r="K70">
-        <v>2.1389999999999998</v>
+        <v>2.139</v>
       </c>
       <c r="L70">
         <v>-0.38</v>
@@ -5095,7 +5060,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21">
       <c r="A71" t="s">
         <v>23</v>
       </c>
@@ -5106,10 +5071,10 @@
         <v>33</v>
       </c>
       <c r="D71">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E71">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="F71">
         <v>0.308</v>
@@ -5127,13 +5092,13 @@
         <v>13</v>
       </c>
       <c r="K71">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L71">
         <v>-0.02</v>
       </c>
       <c r="M71">
-        <v>5.0999999999999997E-2</v>
+        <v>0.051</v>
       </c>
       <c r="N71">
         <v>0.254</v>
@@ -5160,7 +5125,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21">
       <c r="A72" t="s">
         <v>23</v>
       </c>
@@ -5171,13 +5136,13 @@
         <v>36</v>
       </c>
       <c r="D72">
-        <v>0.46200000000000002</v>
+        <v>0.462</v>
       </c>
       <c r="E72">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F72">
-        <v>5.8999999999999997E-2</v>
+        <v>0.059</v>
       </c>
       <c r="G72">
         <v>38</v>
@@ -5192,10 +5157,10 @@
         <v>17</v>
       </c>
       <c r="K72">
-        <v>-1.9E-2</v>
+        <v>-0.019</v>
       </c>
       <c r="L72">
-        <v>-1.4610000000000001</v>
+        <v>-1.461</v>
       </c>
       <c r="M72">
         <v>-1.569</v>
@@ -5225,7 +5190,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:21">
       <c r="A73" t="s">
         <v>23</v>
       </c>
@@ -5236,13 +5201,13 @@
         <v>33</v>
       </c>
       <c r="D73">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="E73">
         <v>0.4</v>
       </c>
       <c r="F73">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="G73">
         <v>31</v>
@@ -5260,13 +5225,13 @@
         <v>-2.14</v>
       </c>
       <c r="L73">
-        <v>0.77200000000000002</v>
+        <v>0.772</v>
       </c>
       <c r="M73">
         <v>0.373</v>
       </c>
       <c r="N73">
-        <v>0.56599999999999995</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="O73" t="s">
         <v>45</v>
@@ -5290,7 +5255,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21">
       <c r="A74" t="s">
         <v>23</v>
       </c>
@@ -5304,10 +5269,10 @@
         <v>0.214</v>
       </c>
       <c r="E74">
-        <v>5.6000000000000001E-2</v>
+        <v>0.056</v>
       </c>
       <c r="F74">
-        <v>0.41199999999999998</v>
+        <v>0.412</v>
       </c>
       <c r="G74">
         <v>30</v>
@@ -5325,10 +5290,10 @@
         <v>-1.665</v>
       </c>
       <c r="L74">
-        <v>-1.4610000000000001</v>
+        <v>-1.461</v>
       </c>
       <c r="M74">
-        <v>0.72799999999999998</v>
+        <v>0.728</v>
       </c>
       <c r="N74">
         <v>0.879</v>
@@ -5355,7 +5320,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21">
       <c r="A75" t="s">
         <v>23</v>
       </c>
@@ -5366,7 +5331,7 @@
         <v>24</v>
       </c>
       <c r="D75">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="E75">
         <v>0.5</v>
@@ -5387,7 +5352,7 @@
         <v>9</v>
       </c>
       <c r="K75">
-        <v>-0.71399999999999997</v>
+        <v>-0.714</v>
       </c>
       <c r="L75">
         <v>1.421</v>
@@ -5420,7 +5385,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21">
       <c r="A76" t="s">
         <v>23</v>
       </c>
@@ -5452,16 +5417,16 @@
         <v>16</v>
       </c>
       <c r="K76">
-        <v>0.90300000000000002</v>
+        <v>0.903</v>
       </c>
       <c r="L76">
         <v>-1.101</v>
       </c>
       <c r="M76">
-        <v>8.2000000000000003E-2</v>
+        <v>0.082</v>
       </c>
       <c r="N76">
-        <v>0.56599999999999995</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="O76" t="s">
         <v>46</v>
@@ -5485,7 +5450,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21">
       <c r="A77" t="s">
         <v>23</v>
       </c>
@@ -5496,13 +5461,13 @@
         <v>27</v>
       </c>
       <c r="D77">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="E77">
-        <v>0.29399999999999998</v>
+        <v>0.294</v>
       </c>
       <c r="F77">
-        <v>0.23100000000000001</v>
+        <v>0.231</v>
       </c>
       <c r="G77">
         <v>35</v>
@@ -5517,16 +5482,16 @@
         <v>13</v>
       </c>
       <c r="K77">
-        <v>-1.1890000000000001</v>
+        <v>-1.189</v>
       </c>
       <c r="L77">
-        <v>8.5999999999999993E-2</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="M77">
         <v>-0.45</v>
       </c>
       <c r="N77">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O77" t="s">
         <v>45</v>
@@ -5550,7 +5515,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21">
       <c r="A78" t="s">
         <v>23</v>
       </c>
@@ -5561,7 +5526,7 @@
         <v>33</v>
       </c>
       <c r="D78">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E78">
         <v>0.312</v>
@@ -5582,16 +5547,16 @@
         <v>13</v>
       </c>
       <c r="K78">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L78">
-        <v>0.20499999999999999</v>
+        <v>0.205</v>
       </c>
       <c r="M78">
         <v>-0.95</v>
       </c>
       <c r="N78">
-        <v>-0.68400000000000005</v>
+        <v>-0.6840000000000001</v>
       </c>
       <c r="O78" t="s">
         <v>44</v>
@@ -5615,7 +5580,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21">
       <c r="A79" t="s">
         <v>23</v>
       </c>
@@ -5626,13 +5591,13 @@
         <v>29</v>
       </c>
       <c r="D79">
-        <v>0.73299999999999998</v>
+        <v>0.733</v>
       </c>
       <c r="E79">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="F79">
-        <v>0.58299999999999996</v>
+        <v>0.583</v>
       </c>
       <c r="G79">
         <v>29</v>
@@ -5653,10 +5618,10 @@
         <v>0.34</v>
       </c>
       <c r="M79">
-        <v>1.8440000000000001</v>
+        <v>1.844</v>
       </c>
       <c r="N79">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="O79" t="s">
         <v>46</v>
@@ -5680,7 +5645,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21">
       <c r="A80" t="s">
         <v>23</v>
       </c>
@@ -5691,13 +5656,13 @@
         <v>34</v>
       </c>
       <c r="D80">
-        <v>0.69199999999999995</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="E80">
         <v>0.5</v>
       </c>
       <c r="F80">
-        <v>0.33300000000000002</v>
+        <v>0.333</v>
       </c>
       <c r="G80">
         <v>36</v>
@@ -5712,7 +5677,7 @@
         <v>9</v>
       </c>
       <c r="K80">
-        <v>1.5169999999999999</v>
+        <v>1.517</v>
       </c>
       <c r="L80">
         <v>1.421</v>
@@ -5745,7 +5710,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21">
       <c r="A81" t="s">
         <v>23</v>
       </c>
@@ -5756,10 +5721,10 @@
         <v>35</v>
       </c>
       <c r="D81">
-        <v>0.42899999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="E81">
-        <v>0.44400000000000001</v>
+        <v>0.444</v>
       </c>
       <c r="F81">
         <v>0.1</v>
@@ -5777,13 +5742,13 @@
         <v>10</v>
       </c>
       <c r="K81">
-        <v>-0.23799999999999999</v>
+        <v>-0.238</v>
       </c>
       <c r="L81">
-        <v>1.0609999999999999</v>
+        <v>1.061</v>
       </c>
       <c r="M81">
-        <v>-1.3009999999999999</v>
+        <v>-1.301</v>
       </c>
       <c r="N81">
         <v>-1.621</v>

</xml_diff>